<commit_message>
Update anomaly test data files for performance history v2.5
</commit_message>
<xml_diff>
--- a/tests/perf_v2/perf_history/v2.5/anomaly/ANOMALY-aggregated.xlsx
+++ b/tests/perf_v2/perf_history/v2.5/anomaly/ANOMALY-aggregated.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AC4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -588,10 +588,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12.5311</v>
+        <v>12.6999</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1003</v>
+        <v>0.1411</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -600,10 +600,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0342</v>
+        <v>0.1907</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0012</v>
+        <v>0.0049</v>
       </c>
       <c r="H2" t="n">
         <v>0.9</v>
@@ -612,16 +612,16 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7941</v>
+        <v>0.794</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0065</v>
+        <v>0.0059</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7835</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0094</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -630,28 +630,28 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0168</v>
+        <v>0.0155</v>
       </c>
       <c r="Q2" t="n">
         <v>0.0002</v>
       </c>
       <c r="R2" t="n">
-        <v>0.07779999999999999</v>
+        <v>0.0543</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0008</v>
+        <v>0.0004</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0644</v>
+        <v>0.0411</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="V2" t="n">
-        <v>28.9768</v>
+        <v>18.5122</v>
       </c>
       <c r="W2" t="n">
-        <v>0.3161</v>
+        <v>0.103</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -670,12 +670,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -691,70 +691,70 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>41.4617</v>
+        <v>641.7163</v>
       </c>
       <c r="C3" t="n">
-        <v>2.4658</v>
+        <v>91.5001</v>
       </c>
       <c r="D3" t="n">
-        <v>5.2</v>
+        <v>59.8</v>
       </c>
       <c r="E3" t="n">
-        <v>0.4472</v>
+        <v>8.671799999999999</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0187</v>
+        <v>0.0238</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0015</v>
+        <v>0.0001</v>
       </c>
       <c r="H3" t="n">
-        <v>1.758</v>
+        <v>1.706</v>
       </c>
       <c r="I3" t="n">
-        <v>0.011</v>
+        <v>0.0456</v>
       </c>
       <c r="J3" t="n">
-        <v>0.7554999999999999</v>
+        <v>0.8338</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0063</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7595</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0018</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.4327</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.3958</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0181</v>
+        <v>0.0151</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0024</v>
+        <v>0.0001</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0712</v>
+        <v>0.0454</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0004</v>
+        <v>0.0007</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0607</v>
+        <v>0.035</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0011</v>
+        <v>0.0005</v>
       </c>
       <c r="V3" t="n">
-        <v>27.3294</v>
+        <v>15.7398</v>
       </c>
       <c r="W3" t="n">
-        <v>0.4768</v>
+        <v>0.2281</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -773,15 +773,118 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
+        <is>
+          <t>tiny</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>uflow</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>972.6434</v>
+      </c>
+      <c r="C4" t="n">
+        <v>10.3453</v>
+      </c>
+      <c r="D4" t="n">
+        <v>199</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0983</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.286</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1399</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.7724</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0111</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0242</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.08749999999999999</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.0183</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0731</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="V4" t="n">
+        <v>32.8828</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.364</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>2.5.0dev</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>ANOMALY</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>mvtec_cable_tiny</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>tiny</t>
         </is>
@@ -798,7 +901,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AC4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -955,10 +1058,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.5607</v>
+        <v>11.3751</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1034</v>
+        <v>0.1757</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -967,58 +1070,58 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0338</v>
+        <v>0.1875</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0005</v>
+        <v>0.0011</v>
       </c>
       <c r="H2" t="n">
-        <v>0.9</v>
+        <v>0.896</v>
       </c>
       <c r="I2" t="n">
-        <v>0</v>
+        <v>0.0089</v>
       </c>
       <c r="J2" t="n">
-        <v>0.9301</v>
+        <v>0.9293</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0017</v>
+        <v>0.0024</v>
       </c>
       <c r="L2" t="n">
-        <v>0.9254</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0117</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0.9082</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0.0189</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0173</v>
+        <v>0.0154</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0004</v>
+        <v>0.0001</v>
       </c>
       <c r="R2" t="n">
-        <v>0.079</v>
+        <v>0.0558</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0004</v>
+        <v>0.0003</v>
       </c>
       <c r="T2" t="n">
-        <v>0.0665</v>
+        <v>0.0434</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0008</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="V2" t="n">
-        <v>26.316</v>
+        <v>17.1858</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2989</v>
+        <v>0.2224</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1037,12 +1140,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -1058,97 +1161,200 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35.0825</v>
+        <v>515.6468</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4604</v>
+        <v>14.5055</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>55.4</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1.6733</v>
       </c>
       <c r="F3" t="n">
-        <v>0.018</v>
+        <v>0.0239</v>
       </c>
       <c r="G3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="H3" t="n">
+        <v>1.604</v>
+      </c>
+      <c r="I3" t="n">
+        <v>0.0378</v>
+      </c>
+      <c r="J3" t="n">
+        <v>0.9054</v>
+      </c>
+      <c r="K3" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="L3" t="n">
+        <v>0</v>
+      </c>
+      <c r="M3" t="n">
+        <v>0</v>
+      </c>
+      <c r="N3" t="n">
+        <v>0</v>
+      </c>
+      <c r="O3" t="n">
+        <v>0</v>
+      </c>
+      <c r="P3" t="n">
+        <v>0.0146</v>
+      </c>
+      <c r="Q3" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.0465</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0359</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.0017</v>
+      </c>
+      <c r="V3" t="n">
+        <v>14.2237</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.6842</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>2.5.0dev</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>ANOMALY</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>mvtec_capsule_tiny</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>tiny</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>uflow</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>889.3396</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7.7287</v>
+      </c>
+      <c r="D4" t="n">
+        <v>199</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0989</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.07</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1434</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.9278</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0136</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0187</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.0805</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.0016</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0742</v>
+      </c>
+      <c r="U4" t="n">
         <v>0.0011</v>
       </c>
-      <c r="H3" t="n">
-        <v>1.778</v>
-      </c>
-      <c r="I3" t="n">
-        <v>0.0217</v>
-      </c>
-      <c r="J3" t="n">
-        <v>0.9008</v>
-      </c>
-      <c r="K3" t="n">
-        <v>0.0017</v>
-      </c>
-      <c r="L3" t="n">
-        <v>0.9026999999999999</v>
-      </c>
-      <c r="M3" t="n">
-        <v>0.0025</v>
-      </c>
-      <c r="N3" t="n">
-        <v>0.3501</v>
-      </c>
-      <c r="O3" t="n">
-        <v>0.4796</v>
-      </c>
-      <c r="P3" t="n">
-        <v>0.013</v>
-      </c>
-      <c r="Q3" t="n">
-        <v>0.0013</v>
-      </c>
-      <c r="R3" t="n">
-        <v>0.07290000000000001</v>
-      </c>
-      <c r="S3" t="n">
-        <v>0.0013</v>
-      </c>
-      <c r="T3" t="n">
-        <v>0.063</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.0007</v>
-      </c>
-      <c r="V3" t="n">
-        <v>24.9373</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.27</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="V4" t="n">
+        <v>29.3658</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.4158</v>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>2.5.0dev</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>ANOMALY</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>mvtec_capsule_tiny</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>release/2.5</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>5a3348332</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>tiny</t>
         </is>
@@ -1165,7 +1371,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AC4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1322,10 +1528,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>12.4906</v>
+        <v>12.2262</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1012</v>
+        <v>0.0482</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -1334,10 +1540,10 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0408</v>
+        <v>0.2104</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0025</v>
+        <v>0.008800000000000001</v>
       </c>
       <c r="H2" t="n">
         <v>0.9</v>
@@ -1346,16 +1552,16 @@
         <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8895999999999999</v>
+        <v>0.8752</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0315</v>
+        <v>0.0304</v>
       </c>
       <c r="L2" t="n">
-        <v>0.8862</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0322</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
         <v>0</v>
@@ -1364,28 +1570,28 @@
         <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0186</v>
+        <v>0.0166</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0003</v>
+        <v>0.0002</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0784</v>
+        <v>0.0554</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0015</v>
+        <v>0.0007</v>
       </c>
       <c r="T2" t="n">
-        <v>0.066</v>
+        <v>0.043</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0008</v>
+        <v>0.0004</v>
       </c>
       <c r="V2" t="n">
-        <v>21.7928</v>
+        <v>14.1743</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2788</v>
+        <v>0.1475</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1404,12 +1610,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -1425,97 +1631,200 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>35.009</v>
+        <v>246.7209</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8135</v>
+        <v>26.4264</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>25.2</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>2.7749</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0755</v>
+        <v>0.2114</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0083</v>
+        <v>0.0015</v>
       </c>
       <c r="H3" t="n">
-        <v>1.768</v>
+        <v>1.656</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0536</v>
+        <v>0.0351</v>
       </c>
       <c r="J3" t="n">
-        <v>0.9018</v>
+        <v>0.9522</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0372</v>
+        <v>0.0151</v>
       </c>
       <c r="L3" t="n">
-        <v>0.8828</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0556</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.1477</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.3304</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0128</v>
+        <v>0.0156</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0003</v>
+        <v>0.0001</v>
       </c>
       <c r="R3" t="n">
-        <v>0.07099999999999999</v>
+        <v>0.0459</v>
       </c>
       <c r="S3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0357</v>
+      </c>
+      <c r="U3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="V3" t="n">
+        <v>11.7653</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.0449</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>2.5.0dev</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>ANOMALY</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>mvtec_hazelnut_small</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>uflow</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1169.1567</v>
+      </c>
+      <c r="C4" t="n">
+        <v>7.3138</v>
+      </c>
+      <c r="D4" t="n">
+        <v>199</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2392</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.004</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.344</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.3806</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.9022</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0136</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0212</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0014</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.0791</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.07149999999999999</v>
+      </c>
+      <c r="U4" t="n">
         <v>0.0009</v>
       </c>
-      <c r="T3" t="n">
-        <v>0.0606</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.0015</v>
-      </c>
-      <c r="V3" t="n">
-        <v>20.0038</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.5012</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="V4" t="n">
+        <v>23.5848</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.2893</v>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>2.5.0dev</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>ANOMALY</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>mvtec_hazelnut_small</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>release/2.5</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>5a3348332</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>small</t>
         </is>
@@ -1532,7 +1841,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AC4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1689,10 +1998,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>20.4922</v>
+        <v>21.4222</v>
       </c>
       <c r="C2" t="n">
-        <v>0.07149999999999999</v>
+        <v>0.9681</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -1701,58 +2010,58 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1114</v>
+        <v>0.1746</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0039</v>
+        <v>0.0032</v>
       </c>
       <c r="H2" t="n">
-        <v>0.912</v>
+        <v>0.9</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0164</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8717</v>
+        <v>0.8776</v>
       </c>
       <c r="K2" t="n">
-        <v>0.0118</v>
+        <v>0.008999999999999999</v>
       </c>
       <c r="L2" t="n">
-        <v>0.854</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0015</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0.3393</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0.4647</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0157</v>
+        <v>0.0112</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0003</v>
+        <v>0.0013</v>
       </c>
       <c r="R2" t="n">
-        <v>0.0785</v>
+        <v>0.0554</v>
       </c>
       <c r="S2" t="n">
         <v>0.0007</v>
       </c>
       <c r="T2" t="n">
-        <v>0.066</v>
+        <v>0.0431</v>
       </c>
       <c r="U2" t="n">
         <v>0.0003</v>
       </c>
       <c r="V2" t="n">
-        <v>31.6741</v>
+        <v>20.6878</v>
       </c>
       <c r="W2" t="n">
-        <v>0.1481</v>
+        <v>0.1654</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -1771,12 +2080,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -1792,97 +2101,200 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>68.3228</v>
+        <v>154.5618</v>
       </c>
       <c r="C3" t="n">
-        <v>0.4512</v>
+        <v>24.6611</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>10.4</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>1.8166</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0989</v>
+        <v>0.1728</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0005</v>
+        <v>0.0008</v>
       </c>
       <c r="H3" t="n">
-        <v>1.76</v>
+        <v>1.6</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0212</v>
+        <v>0.0308</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8489</v>
+        <v>0.8618</v>
       </c>
       <c r="K3" t="n">
-        <v>0</v>
+        <v>0.0205</v>
       </c>
       <c r="L3" t="n">
-        <v>0.853</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
         <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.853</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0104</v>
+        <v>0.0098</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0005</v>
+        <v>0.0002</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0713</v>
+        <v>0.0466</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0007</v>
+        <v>0.0003</v>
       </c>
       <c r="T3" t="n">
-        <v>0.061</v>
+        <v>0.034</v>
       </c>
       <c r="U3" t="n">
+        <v>0.0003</v>
+      </c>
+      <c r="V3" t="n">
+        <v>16.328</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.157</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>2.5.0dev</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>ANOMALY</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>mvtec_screw_medium</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>uflow</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>2833.7768</v>
+      </c>
+      <c r="C4" t="n">
+        <v>22.9764</v>
+      </c>
+      <c r="D4" t="n">
+        <v>199</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2023</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0012</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.094</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1374</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.8582</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.007</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0153</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.0771</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.001</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0683</v>
+      </c>
+      <c r="U4" t="n">
         <v>0.0004</v>
       </c>
-      <c r="V3" t="n">
-        <v>29.2709</v>
-      </c>
-      <c r="W3" t="n">
-        <v>0.2094</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="V4" t="n">
+        <v>32.7699</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.1851</v>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>2.5.0dev</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>ANOMALY</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>mvtec_screw_medium</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>release/2.5</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>5a3348332</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
@@ -1899,7 +2311,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AC4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2056,10 +2468,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>11.5382</v>
+        <v>11.2828</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1267</v>
+        <v>0.1836</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -2068,58 +2480,58 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.0387</v>
+        <v>0.139</v>
       </c>
       <c r="G2" t="n">
+        <v>0.0089</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.8028</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.027</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.0182</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.0552</v>
+      </c>
+      <c r="S2" t="n">
         <v>0.0004</v>
       </c>
-      <c r="H2" t="n">
-        <v>0.906</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.0134</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.8198</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.035</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.7816</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.0512</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.3148</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.4316</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.0191</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.0788</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.0003</v>
-      </c>
       <c r="T2" t="n">
-        <v>0.0655</v>
+        <v>0.0426</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0005</v>
+        <v>0.0009</v>
       </c>
       <c r="V2" t="n">
-        <v>19.6484</v>
+        <v>12.7757</v>
       </c>
       <c r="W2" t="n">
-        <v>0.1479</v>
+        <v>0.2552</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -2138,12 +2550,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -2159,70 +2571,70 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>30.9076</v>
+        <v>283.7912</v>
       </c>
       <c r="C3" t="n">
-        <v>0.1226</v>
+        <v>53.8974</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>30.4</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>6.0249</v>
       </c>
       <c r="F3" t="n">
-        <v>0.0536</v>
+        <v>0.1299</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0024</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="H3" t="n">
-        <v>1.744</v>
+        <v>1.644</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0152</v>
+        <v>0.0251</v>
       </c>
       <c r="J3" t="n">
-        <v>0.5678</v>
+        <v>0.7623</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0109</v>
+        <v>0.0232</v>
       </c>
       <c r="L3" t="n">
-        <v>0.5648</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.009599999999999999</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.2286</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
-        <v>0.313</v>
+        <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0.0146</v>
+        <v>0.0175</v>
       </c>
       <c r="Q3" t="n">
-        <v>0.0025</v>
+        <v>0.0005</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0721</v>
+        <v>0.0455</v>
       </c>
       <c r="S3" t="n">
-        <v>0.0007</v>
+        <v>0.0002</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0635</v>
+        <v>0.0358</v>
       </c>
       <c r="U3" t="n">
         <v>0.0003</v>
       </c>
       <c r="V3" t="n">
-        <v>19.0404</v>
+        <v>10.7446</v>
       </c>
       <c r="W3" t="n">
-        <v>0.0866</v>
+        <v>0.0992</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -2241,15 +2653,118 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
+        <is>
+          <t>small</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>uflow</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>1068.673</v>
+      </c>
+      <c r="C4" t="n">
+        <v>4.8959</v>
+      </c>
+      <c r="D4" t="n">
+        <v>199</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.1581</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0023</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.298</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1272</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.6984</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0317</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.0284</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0015</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.078</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.0721</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="V4" t="n">
+        <v>21.6348</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.3392</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>2.5.0dev</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>ANOMALY</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>mvtec_transistor_small</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>small</t>
         </is>
@@ -2266,7 +2781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AC4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2423,10 +2938,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>28.5173</v>
+        <v>28.7455</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1642</v>
+        <v>0.1539</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -2435,58 +2950,58 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.1757</v>
+        <v>0.1833</v>
       </c>
       <c r="G2" t="n">
-        <v>0.0031</v>
+        <v>0.0012</v>
       </c>
       <c r="H2" t="n">
-        <v>0.924</v>
+        <v>0.93</v>
       </c>
       <c r="I2" t="n">
-        <v>0.0134</v>
+        <v>0</v>
       </c>
       <c r="J2" t="n">
-        <v>0.7755</v>
+        <v>0.7731</v>
       </c>
       <c r="K2" t="n">
         <v>0.0068</v>
       </c>
       <c r="L2" t="n">
-        <v>0.7698</v>
+        <v>0</v>
       </c>
       <c r="M2" t="n">
-        <v>0.0017</v>
+        <v>0</v>
       </c>
       <c r="N2" t="n">
-        <v>0.6114000000000001</v>
+        <v>0</v>
       </c>
       <c r="O2" t="n">
-        <v>0.3419</v>
+        <v>0</v>
       </c>
       <c r="P2" t="n">
-        <v>0.0162</v>
+        <v>0.0097</v>
       </c>
       <c r="Q2" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0002</v>
       </c>
       <c r="R2" t="n">
-        <v>0.08309999999999999</v>
+        <v>0.059</v>
       </c>
       <c r="S2" t="n">
-        <v>0.0008</v>
+        <v>0.0005</v>
       </c>
       <c r="T2" t="n">
-        <v>0.07199999999999999</v>
+        <v>0.0466</v>
       </c>
       <c r="U2" t="n">
-        <v>0.0018</v>
+        <v>0.0003</v>
       </c>
       <c r="V2" t="n">
-        <v>34.5394</v>
+        <v>22.379</v>
       </c>
       <c r="W2" t="n">
-        <v>0.8804999999999999</v>
+        <v>0.1586</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -2505,12 +3020,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -2526,97 +3041,200 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>104.2645</v>
+        <v>265.1049</v>
       </c>
       <c r="C3" t="n">
-        <v>0.6522</v>
+        <v>62.2054</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>13.4</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>3.3615</v>
       </c>
       <c r="F3" t="n">
-        <v>0.1715</v>
+        <v>0.1932</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0005</v>
+        <v>0.0072</v>
       </c>
       <c r="H3" t="n">
-        <v>1.782</v>
+        <v>1.612</v>
       </c>
       <c r="I3" t="n">
-        <v>0.0402</v>
+        <v>0.0217</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8169999999999999</v>
+        <v>0.8246</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0166</v>
+        <v>0.0146</v>
       </c>
       <c r="L3" t="n">
-        <v>0.7683</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0021</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.7692</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
       </c>
       <c r="P3" t="n">
-        <v>0.009900000000000001</v>
+        <v>0.0095</v>
       </c>
       <c r="Q3" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="R3" t="n">
+        <v>0.0494</v>
+      </c>
+      <c r="S3" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="T3" t="n">
+        <v>0.0396</v>
+      </c>
+      <c r="U3" t="n">
         <v>0.0003</v>
       </c>
-      <c r="R3" t="n">
-        <v>0.078</v>
-      </c>
-      <c r="S3" t="n">
+      <c r="V3" t="n">
+        <v>18.9863</v>
+      </c>
+      <c r="W3" t="n">
+        <v>0.1273</v>
+      </c>
+      <c r="X3" t="inlineStr">
+        <is>
+          <t>2.5.0dev</t>
+        </is>
+      </c>
+      <c r="Y3" t="inlineStr">
+        <is>
+          <t>ANOMALY</t>
+        </is>
+      </c>
+      <c r="Z3" t="inlineStr">
+        <is>
+          <t>visa_capsules_medium</t>
+        </is>
+      </c>
+      <c r="AA3" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB3" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC3" t="inlineStr">
+        <is>
+          <t>medium</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>uflow</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>5221.9115</v>
+      </c>
+      <c r="C4" t="n">
+        <v>47.2122</v>
+      </c>
+      <c r="D4" t="n">
+        <v>199</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.2192</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0029</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.452</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.1524</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.7891</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.005</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.014</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0007</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.0795</v>
+      </c>
+      <c r="S4" t="n">
         <v>0.0005999999999999999</v>
       </c>
-      <c r="T3" t="n">
-        <v>0.0709</v>
-      </c>
-      <c r="U3" t="n">
-        <v>0.0026</v>
-      </c>
-      <c r="V3" t="n">
-        <v>34.054</v>
-      </c>
-      <c r="W3" t="n">
-        <v>1.2446</v>
-      </c>
-      <c r="X3" t="inlineStr">
+      <c r="T4" t="n">
+        <v>0.0706</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.0011</v>
+      </c>
+      <c r="V4" t="n">
+        <v>33.9063</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.5127</v>
+      </c>
+      <c r="X4" t="inlineStr">
         <is>
           <t>2.5.0dev</t>
         </is>
       </c>
-      <c r="Y3" t="inlineStr">
+      <c r="Y4" t="inlineStr">
         <is>
           <t>ANOMALY</t>
         </is>
       </c>
-      <c r="Z3" t="inlineStr">
+      <c r="Z4" t="inlineStr">
         <is>
           <t>visa_capsules_medium</t>
         </is>
       </c>
-      <c r="AA3" t="inlineStr">
-        <is>
-          <t>release/2.5</t>
-        </is>
-      </c>
-      <c r="AB3" t="inlineStr">
-        <is>
-          <t>5a3348332</t>
-        </is>
-      </c>
-      <c r="AC3" t="inlineStr">
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>medium</t>
         </is>
@@ -2633,7 +3251,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AC3"/>
+  <dimension ref="A1:AC4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -2790,10 +3408,10 @@
         </is>
       </c>
       <c r="B2" t="n">
-        <v>41.026</v>
+        <v>42.2987</v>
       </c>
       <c r="C2" t="n">
-        <v>0.1313</v>
+        <v>0.197</v>
       </c>
       <c r="D2" t="n">
         <v>0</v>
@@ -2802,58 +3420,58 @@
         <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>0.185</v>
+        <v>0.1869</v>
       </c>
       <c r="G2" t="n">
+        <v>0.0019</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.962</v>
+      </c>
+      <c r="I2" t="n">
+        <v>0.0205</v>
+      </c>
+      <c r="J2" t="n">
+        <v>0.7257</v>
+      </c>
+      <c r="K2" t="n">
+        <v>0.0191</v>
+      </c>
+      <c r="L2" t="n">
+        <v>0</v>
+      </c>
+      <c r="M2" t="n">
+        <v>0</v>
+      </c>
+      <c r="N2" t="n">
+        <v>0</v>
+      </c>
+      <c r="O2" t="n">
+        <v>0</v>
+      </c>
+      <c r="P2" t="n">
+        <v>0.0089</v>
+      </c>
+      <c r="Q2" t="n">
+        <v>0.0001</v>
+      </c>
+      <c r="R2" t="n">
+        <v>0.0578</v>
+      </c>
+      <c r="S2" t="n">
+        <v>0.0002</v>
+      </c>
+      <c r="T2" t="n">
+        <v>0.047</v>
+      </c>
+      <c r="U2" t="n">
         <v>0.0003</v>
       </c>
-      <c r="H2" t="n">
-        <v>0.97</v>
-      </c>
-      <c r="I2" t="n">
-        <v>0.0224</v>
-      </c>
-      <c r="J2" t="n">
-        <v>0.7326</v>
-      </c>
-      <c r="K2" t="n">
-        <v>0.0118</v>
-      </c>
-      <c r="L2" t="n">
-        <v>0.6976</v>
-      </c>
-      <c r="M2" t="n">
-        <v>0.0171</v>
-      </c>
-      <c r="N2" t="n">
-        <v>0.6814</v>
-      </c>
-      <c r="O2" t="n">
-        <v>0.0138</v>
-      </c>
-      <c r="P2" t="n">
-        <v>0.0154</v>
-      </c>
-      <c r="Q2" t="n">
-        <v>0.0003</v>
-      </c>
-      <c r="R2" t="n">
-        <v>0.0828</v>
-      </c>
-      <c r="S2" t="n">
-        <v>0.0014</v>
-      </c>
-      <c r="T2" t="n">
-        <v>0.0755</v>
-      </c>
-      <c r="U2" t="n">
-        <v>0.0005</v>
-      </c>
       <c r="V2" t="n">
-        <v>45.5255</v>
+        <v>28.3419</v>
       </c>
       <c r="W2" t="n">
-        <v>0.2797</v>
+        <v>0.1944</v>
       </c>
       <c r="X2" t="inlineStr">
         <is>
@@ -2872,12 +3490,12 @@
       </c>
       <c r="AA2" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB2" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC2" t="inlineStr">
@@ -2893,43 +3511,43 @@
         </is>
       </c>
       <c r="B3" t="n">
-        <v>155.1261</v>
+        <v>349.1181</v>
       </c>
       <c r="C3" t="n">
-        <v>0.8062</v>
+        <v>53.8007</v>
       </c>
       <c r="D3" t="n">
-        <v>5</v>
+        <v>12</v>
       </c>
       <c r="E3" t="n">
-        <v>0</v>
+        <v>2.1213</v>
       </c>
       <c r="F3" t="n">
-        <v>0.182</v>
+        <v>0.1943</v>
       </c>
       <c r="G3" t="n">
-        <v>0.0011</v>
+        <v>0.0039</v>
       </c>
       <c r="H3" t="n">
-        <v>1.752</v>
+        <v>1.612</v>
       </c>
       <c r="I3" t="n">
-        <v>0.011</v>
+        <v>0.0409</v>
       </c>
       <c r="J3" t="n">
-        <v>0.8165</v>
+        <v>0.8296</v>
       </c>
       <c r="K3" t="n">
-        <v>0.0124</v>
+        <v>0.0438</v>
       </c>
       <c r="L3" t="n">
-        <v>0.673</v>
+        <v>0</v>
       </c>
       <c r="M3" t="n">
-        <v>0.0041</v>
+        <v>0</v>
       </c>
       <c r="N3" t="n">
-        <v>0.6645</v>
+        <v>0</v>
       </c>
       <c r="O3" t="n">
         <v>0</v>
@@ -2941,22 +3559,22 @@
         <v>0.0001</v>
       </c>
       <c r="R3" t="n">
-        <v>0.0774</v>
+        <v>0.0495</v>
       </c>
       <c r="S3" t="n">
-        <v>0.001</v>
+        <v>0.0004</v>
       </c>
       <c r="T3" t="n">
-        <v>0.0716</v>
+        <v>0.0406</v>
       </c>
       <c r="U3" t="n">
-        <v>0.0009</v>
+        <v>0.0003</v>
       </c>
       <c r="V3" t="n">
-        <v>43.1915</v>
+        <v>24.5032</v>
       </c>
       <c r="W3" t="n">
-        <v>0.5128</v>
+        <v>0.1753</v>
       </c>
       <c r="X3" t="inlineStr">
         <is>
@@ -2975,15 +3593,118 @@
       </c>
       <c r="AA3" t="inlineStr">
         <is>
-          <t>release/2.5</t>
+          <t>HEAD</t>
         </is>
       </c>
       <c r="AB3" t="inlineStr">
         <is>
-          <t>5a3348332</t>
+          <t>9b7168126</t>
         </is>
       </c>
       <c r="AC3" t="inlineStr">
+        <is>
+          <t>large</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
+          <t>uflow</t>
+        </is>
+      </c>
+      <c r="B4" t="n">
+        <v>7445.3683</v>
+      </c>
+      <c r="C4" t="n">
+        <v>87.3489</v>
+      </c>
+      <c r="D4" t="n">
+        <v>199</v>
+      </c>
+      <c r="E4" t="n">
+        <v>0</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.222</v>
+      </c>
+      <c r="G4" t="n">
+        <v>0.0043</v>
+      </c>
+      <c r="H4" t="n">
+        <v>6.46</v>
+      </c>
+      <c r="I4" t="n">
+        <v>0.0412</v>
+      </c>
+      <c r="J4" t="n">
+        <v>0.8002</v>
+      </c>
+      <c r="K4" t="n">
+        <v>0.0041</v>
+      </c>
+      <c r="L4" t="n">
+        <v>0</v>
+      </c>
+      <c r="M4" t="n">
+        <v>0</v>
+      </c>
+      <c r="N4" t="n">
+        <v>0</v>
+      </c>
+      <c r="O4" t="n">
+        <v>0</v>
+      </c>
+      <c r="P4" t="n">
+        <v>0.013</v>
+      </c>
+      <c r="Q4" t="n">
+        <v>0.0008</v>
+      </c>
+      <c r="R4" t="n">
+        <v>0.0799</v>
+      </c>
+      <c r="S4" t="n">
+        <v>0.0005999999999999999</v>
+      </c>
+      <c r="T4" t="n">
+        <v>0.07099999999999999</v>
+      </c>
+      <c r="U4" t="n">
+        <v>0.0013</v>
+      </c>
+      <c r="V4" t="n">
+        <v>42.7938</v>
+      </c>
+      <c r="W4" t="n">
+        <v>0.764</v>
+      </c>
+      <c r="X4" t="inlineStr">
+        <is>
+          <t>2.5.0dev</t>
+        </is>
+      </c>
+      <c r="Y4" t="inlineStr">
+        <is>
+          <t>ANOMALY</t>
+        </is>
+      </c>
+      <c r="Z4" t="inlineStr">
+        <is>
+          <t>visa_pcb3_large</t>
+        </is>
+      </c>
+      <c r="AA4" t="inlineStr">
+        <is>
+          <t>HEAD</t>
+        </is>
+      </c>
+      <c r="AB4" t="inlineStr">
+        <is>
+          <t>9b7168126</t>
+        </is>
+      </c>
+      <c r="AC4" t="inlineStr">
         <is>
           <t>large</t>
         </is>

</xml_diff>